<commit_message>
sql: updated revenue logic with actual vs estimated revenue and added revenue loss analysis
</commit_message>
<xml_diff>
--- a/sql_metrics/SQL_Output_Tables.xlsx
+++ b/sql_metrics/SQL_Output_Tables.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
   <si>
     <t>Revenue By Room</t>
   </si>
@@ -26,13 +26,13 @@
     <t>room_type</t>
   </si>
   <si>
-    <t>revenue</t>
+    <t>Estimated Revenue</t>
+  </si>
+  <si>
+    <t>Actual Revenue</t>
   </si>
   <si>
     <t>City</t>
-  </si>
-  <si>
-    <t>Revenue</t>
   </si>
   <si>
     <t>Standard</t>
@@ -284,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -297,14 +297,20 @@
     <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -365,6 +371,9 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="17" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="17" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -598,7 +607,12 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="12.63"/>
+    <col customWidth="1" min="1" max="3" width="12.63"/>
+    <col customWidth="1" min="4" max="4" width="17.88"/>
+    <col customWidth="1" min="5" max="5" width="13.75"/>
+    <col customWidth="1" min="6" max="6" width="12.63"/>
+    <col customWidth="1" min="8" max="8" width="16.75"/>
+    <col customWidth="1" min="9" max="9" width="13.88"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1"/>
@@ -606,7 +620,7 @@
     <row r="3" ht="15.75" customHeight="1"/>
     <row r="4" ht="15.75" customHeight="1"/>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="D5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -614,74 +628,104 @@
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="G6" s="6" t="s">
         <v>5</v>
       </c>
+      <c r="H6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="D7" s="5" t="s">
+      <c r="C7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="6">
+      <c r="D7" s="8">
         <v>1.148344E7</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="E7" s="8">
+        <v>5293695.0</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="9">
         <v>7231831.0</v>
       </c>
+      <c r="I7" s="9">
+        <v>7231831.0</v>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="6">
+      <c r="D8" s="8">
+        <v>1.1380601E7</v>
+      </c>
+      <c r="E8" s="8">
+        <v>4970937.0</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" s="9">
+        <v>6672277.0</v>
+      </c>
+      <c r="I8" s="9">
+        <v>7136611.0</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="C9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="8">
         <v>1.1452622E7</v>
       </c>
-      <c r="G8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="H8" s="7">
+      <c r="E9" s="8">
+        <v>4623389.0</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="9">
         <v>7136611.0</v>
       </c>
-    </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="D9" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="6">
-        <v>1.1380601E7</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="H9" s="7">
+      <c r="I9" s="9">
         <v>6935673.0</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="9">
+        <v>6935673.0</v>
+      </c>
+      <c r="I10" s="9">
         <v>6672277.0</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="9">
+        <v>6340271.0</v>
+      </c>
+      <c r="I11" s="9">
         <v>6340271.0</v>
       </c>
     </row>
@@ -1676,8 +1720,8 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="C5:E5"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1699,171 +1743,171 @@
     <row r="4" ht="15.75" customHeight="1"/>
     <row r="5" ht="15.75" customHeight="1"/>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="I7" s="11" t="s">
+      <c r="H7" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="13" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="E8" s="12">
+      <c r="E8" s="14">
         <v>1.0</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="14">
         <v>171.0</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="14">
+      <c r="I8" s="16">
         <v>420.0</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="E9" s="12">
+      <c r="E9" s="14">
         <v>2.0</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="14">
         <v>151.0</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="I9" s="14">
+      <c r="I9" s="16">
         <v>419.0</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="E10" s="12">
+      <c r="E10" s="14">
         <v>3.0</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="14">
         <v>168.0</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="14">
+      <c r="I10" s="16">
         <v>399.0</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="E11" s="12">
+      <c r="E11" s="14">
         <v>4.0</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="14">
         <v>177.0</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="I11" s="14">
+      <c r="I11" s="16">
         <v>387.0</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="E12" s="12">
+      <c r="E12" s="14">
         <v>5.0</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="14">
         <v>192.0</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="I12" s="14">
+      <c r="I12" s="16">
         <v>375.0</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="E13" s="12">
+      <c r="E13" s="14">
         <v>6.0</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="14">
         <v>174.0</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="E14" s="12">
+      <c r="E14" s="14">
         <v>7.0</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="14">
         <v>146.0</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="E15" s="12">
+      <c r="E15" s="14">
         <v>8.0</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="14">
         <v>165.0</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="17" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="E16" s="12">
+      <c r="E16" s="14">
         <v>9.0</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="14">
         <v>165.0</v>
       </c>
-      <c r="H16" s="16" t="s">
+      <c r="H16" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="16" t="s">
+      <c r="I16" s="18" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="E17" s="12">
+      <c r="E17" s="14">
         <v>10.0</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="14">
         <v>177.0</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="20">
         <v>989.0</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="E18" s="12">
+      <c r="E18" s="14">
         <v>11.0</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="14">
         <v>151.0</v>
       </c>
-      <c r="H18" s="17" t="s">
+      <c r="H18" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="18">
+      <c r="I18" s="20">
         <v>1011.0</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="E19" s="12">
+      <c r="E19" s="14">
         <v>12.0</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="14">
         <v>163.0</v>
       </c>
     </row>
@@ -2875,1277 +2919,1277 @@
     <row r="4" ht="15.75" customHeight="1"/>
     <row r="5" ht="15.75" customHeight="1"/>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="21" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="22" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="G8" s="21">
+      <c r="G8" s="23">
         <v>1.0</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="23">
         <v>0.2571</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="G9" s="21">
+      <c r="G9" s="23">
         <v>2.0</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="23">
         <v>0.2963</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="G10" s="21">
+      <c r="G10" s="23">
         <v>3.0</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="23">
         <v>0.2973</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="G11" s="21">
+      <c r="G11" s="23">
         <v>4.0</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="23">
         <v>0.2059</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="G12" s="21">
+      <c r="G12" s="23">
         <v>5.0</v>
       </c>
-      <c r="H12" s="21">
+      <c r="H12" s="23">
         <v>0.3226</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="G13" s="21">
+      <c r="G13" s="23">
         <v>6.0</v>
       </c>
-      <c r="H13" s="21">
+      <c r="H13" s="23">
         <v>0.2258</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="G14" s="21">
+      <c r="G14" s="23">
         <v>7.0</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="23">
         <v>0.2727</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="G15" s="21">
+      <c r="G15" s="23">
         <v>8.0</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="23">
         <v>0.2857</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="G16" s="21">
+      <c r="G16" s="23">
         <v>9.0</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="23">
         <v>0.3448</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="G17" s="21">
+      <c r="G17" s="23">
         <v>10.0</v>
       </c>
-      <c r="H17" s="21">
+      <c r="H17" s="23">
         <v>0.4118</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="G18" s="21">
+      <c r="G18" s="23">
         <v>11.0</v>
       </c>
-      <c r="H18" s="21">
+      <c r="H18" s="23">
         <v>0.2903</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="G19" s="21">
+      <c r="G19" s="23">
         <v>12.0</v>
       </c>
-      <c r="H19" s="21">
+      <c r="H19" s="23">
         <v>0.4839</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="G20" s="21">
+      <c r="G20" s="23">
         <v>13.0</v>
       </c>
-      <c r="H20" s="21">
+      <c r="H20" s="23">
         <v>0.3846</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="G21" s="21">
+      <c r="G21" s="23">
         <v>14.0</v>
       </c>
-      <c r="H21" s="21">
+      <c r="H21" s="23">
         <v>0.36</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="G22" s="21">
+      <c r="G22" s="23">
         <v>15.0</v>
       </c>
-      <c r="H22" s="21">
+      <c r="H22" s="23">
         <v>0.5526</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="G23" s="21">
+      <c r="G23" s="23">
         <v>16.0</v>
       </c>
-      <c r="H23" s="21">
+      <c r="H23" s="23">
         <v>0.4667</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="G24" s="21">
+      <c r="G24" s="23">
         <v>17.0</v>
       </c>
-      <c r="H24" s="21">
+      <c r="H24" s="23">
         <v>0.4043</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="G25" s="21">
+      <c r="G25" s="23">
         <v>18.0</v>
       </c>
-      <c r="H25" s="21">
+      <c r="H25" s="23">
         <v>0.5172</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="G26" s="21">
+      <c r="G26" s="23">
         <v>19.0</v>
       </c>
-      <c r="H26" s="21">
+      <c r="H26" s="23">
         <v>0.5833</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="G27" s="21">
+      <c r="G27" s="23">
         <v>20.0</v>
       </c>
-      <c r="H27" s="21">
+      <c r="H27" s="23">
         <v>0.3846</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="G28" s="21">
+      <c r="G28" s="23">
         <v>21.0</v>
       </c>
-      <c r="H28" s="21">
+      <c r="H28" s="23">
         <v>0.4571</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="G29" s="21">
+      <c r="G29" s="23">
         <v>22.0</v>
       </c>
-      <c r="H29" s="21">
+      <c r="H29" s="23">
         <v>0.4634</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="G30" s="21">
+      <c r="G30" s="23">
         <v>23.0</v>
       </c>
-      <c r="H30" s="21">
+      <c r="H30" s="23">
         <v>0.5429</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="G31" s="21">
+      <c r="G31" s="23">
         <v>24.0</v>
       </c>
-      <c r="H31" s="21">
+      <c r="H31" s="23">
         <v>0.4286</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="G32" s="21">
+      <c r="G32" s="23">
         <v>25.0</v>
       </c>
-      <c r="H32" s="21">
+      <c r="H32" s="23">
         <v>0.3636</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="G33" s="21">
+      <c r="G33" s="23">
         <v>26.0</v>
       </c>
-      <c r="H33" s="21">
+      <c r="H33" s="23">
         <v>0.5938</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="G34" s="21">
+      <c r="G34" s="23">
         <v>27.0</v>
       </c>
-      <c r="H34" s="21">
+      <c r="H34" s="23">
         <v>0.5</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="G35" s="21">
+      <c r="G35" s="23">
         <v>28.0</v>
       </c>
-      <c r="H35" s="21">
+      <c r="H35" s="23">
         <v>0.5833</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="G36" s="21">
+      <c r="G36" s="23">
         <v>29.0</v>
       </c>
-      <c r="H36" s="21">
+      <c r="H36" s="23">
         <v>0.6667</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="G37" s="21">
+      <c r="G37" s="23">
         <v>30.0</v>
       </c>
-      <c r="H37" s="21">
+      <c r="H37" s="23">
         <v>0.4706</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="G38" s="21">
+      <c r="G38" s="23">
         <v>31.0</v>
       </c>
-      <c r="H38" s="21">
+      <c r="H38" s="23">
         <v>0.7037</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="G39" s="21">
+      <c r="G39" s="23">
         <v>32.0</v>
       </c>
-      <c r="H39" s="21">
+      <c r="H39" s="23">
         <v>0.525</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="G40" s="21">
+      <c r="G40" s="23">
         <v>33.0</v>
       </c>
-      <c r="H40" s="21">
+      <c r="H40" s="23">
         <v>0.5417</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="G41" s="21">
+      <c r="G41" s="23">
         <v>34.0</v>
       </c>
-      <c r="H41" s="21">
+      <c r="H41" s="23">
         <v>0.5714</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="G42" s="21">
+      <c r="G42" s="23">
         <v>35.0</v>
       </c>
-      <c r="H42" s="21">
+      <c r="H42" s="23">
         <v>0.5152</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="G43" s="21">
+      <c r="G43" s="23">
         <v>36.0</v>
       </c>
-      <c r="H43" s="21">
+      <c r="H43" s="23">
         <v>0.6071</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="G44" s="21">
+      <c r="G44" s="23">
         <v>37.0</v>
       </c>
-      <c r="H44" s="21">
+      <c r="H44" s="23">
         <v>0.6207</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="G45" s="21">
+      <c r="G45" s="23">
         <v>38.0</v>
       </c>
-      <c r="H45" s="21">
+      <c r="H45" s="23">
         <v>0.6667</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="G46" s="21">
+      <c r="G46" s="23">
         <v>39.0</v>
       </c>
-      <c r="H46" s="21">
+      <c r="H46" s="23">
         <v>0.5667</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="G47" s="21">
+      <c r="G47" s="23">
         <v>40.0</v>
       </c>
-      <c r="H47" s="21">
+      <c r="H47" s="23">
         <v>0.6047</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="G48" s="21">
+      <c r="G48" s="23">
         <v>41.0</v>
       </c>
-      <c r="H48" s="21">
+      <c r="H48" s="23">
         <v>0.7308</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="G49" s="21">
+      <c r="G49" s="23">
         <v>42.0</v>
       </c>
-      <c r="H49" s="21">
+      <c r="H49" s="23">
         <v>0.6563</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="G50" s="21">
+      <c r="G50" s="23">
         <v>43.0</v>
       </c>
-      <c r="H50" s="21">
+      <c r="H50" s="23">
         <v>0.6667</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="G51" s="21">
+      <c r="G51" s="23">
         <v>44.0</v>
       </c>
-      <c r="H51" s="21">
+      <c r="H51" s="23">
         <v>0.7037</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="G52" s="21">
+      <c r="G52" s="23">
         <v>45.0</v>
       </c>
-      <c r="H52" s="21">
+      <c r="H52" s="23">
         <v>0.6389</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="G53" s="21">
+      <c r="G53" s="23">
         <v>46.0</v>
       </c>
-      <c r="H53" s="21">
+      <c r="H53" s="23">
         <v>0.7667</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="G54" s="21">
+      <c r="G54" s="23">
         <v>47.0</v>
       </c>
-      <c r="H54" s="21">
+      <c r="H54" s="23">
         <v>0.641</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="G55" s="21">
+      <c r="G55" s="23">
         <v>48.0</v>
       </c>
-      <c r="H55" s="21">
+      <c r="H55" s="23">
         <v>0.675</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="G56" s="21">
+      <c r="G56" s="23">
         <v>49.0</v>
       </c>
-      <c r="H56" s="21">
+      <c r="H56" s="23">
         <v>0.8182</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="G57" s="21">
+      <c r="G57" s="23">
         <v>50.0</v>
       </c>
-      <c r="H57" s="21">
+      <c r="H57" s="23">
         <v>0.7188</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="G58" s="21">
+      <c r="G58" s="23">
         <v>51.0</v>
       </c>
-      <c r="H58" s="21">
+      <c r="H58" s="23">
         <v>0.7</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="G59" s="21">
+      <c r="G59" s="23">
         <v>52.0</v>
       </c>
-      <c r="H59" s="21">
+      <c r="H59" s="23">
         <v>0.8387</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="G60" s="21">
+      <c r="G60" s="23">
         <v>53.0</v>
       </c>
-      <c r="H60" s="21">
+      <c r="H60" s="23">
         <v>0.7778</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="22"/>
-      <c r="B61" s="22"/>
-      <c r="G61" s="21">
+      <c r="A61" s="24"/>
+      <c r="B61" s="24"/>
+      <c r="G61" s="23">
         <v>54.0</v>
       </c>
-      <c r="H61" s="21">
+      <c r="H61" s="23">
         <v>0.8049</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="22"/>
-      <c r="B62" s="22"/>
-      <c r="G62" s="21">
+      <c r="A62" s="24"/>
+      <c r="B62" s="24"/>
+      <c r="G62" s="23">
         <v>55.0</v>
       </c>
-      <c r="H62" s="21">
+      <c r="H62" s="23">
         <v>0.7955</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="22"/>
-      <c r="B63" s="22"/>
-      <c r="G63" s="21">
+      <c r="A63" s="24"/>
+      <c r="B63" s="24"/>
+      <c r="G63" s="23">
         <v>56.0</v>
       </c>
-      <c r="H63" s="21">
+      <c r="H63" s="23">
         <v>0.8108</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="22"/>
-      <c r="B64" s="22"/>
-      <c r="G64" s="21">
+      <c r="A64" s="24"/>
+      <c r="B64" s="24"/>
+      <c r="G64" s="23">
         <v>57.0</v>
       </c>
-      <c r="H64" s="21">
+      <c r="H64" s="23">
         <v>0.7838</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="22"/>
-      <c r="B65" s="22"/>
-      <c r="G65" s="21">
+      <c r="A65" s="24"/>
+      <c r="B65" s="24"/>
+      <c r="G65" s="23">
         <v>58.0</v>
       </c>
-      <c r="H65" s="21">
+      <c r="H65" s="23">
         <v>0.8049</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="22"/>
-      <c r="B66" s="22"/>
-      <c r="G66" s="21">
+      <c r="A66" s="24"/>
+      <c r="B66" s="24"/>
+      <c r="G66" s="23">
         <v>59.0</v>
       </c>
-      <c r="H66" s="21">
+      <c r="H66" s="23">
         <v>0.88</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="22"/>
-      <c r="B67" s="22"/>
+      <c r="A67" s="24"/>
+      <c r="B67" s="24"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="22"/>
-      <c r="B68" s="22"/>
+      <c r="A68" s="24"/>
+      <c r="B68" s="24"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="22"/>
-      <c r="B69" s="22"/>
+      <c r="A69" s="24"/>
+      <c r="B69" s="24"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="22"/>
-      <c r="B70" s="22"/>
+      <c r="A70" s="24"/>
+      <c r="B70" s="24"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="22"/>
-      <c r="B71" s="22"/>
+      <c r="A71" s="24"/>
+      <c r="B71" s="24"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="22"/>
-      <c r="B72" s="22"/>
+      <c r="A72" s="24"/>
+      <c r="B72" s="24"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="22"/>
-      <c r="B73" s="22"/>
+      <c r="A73" s="24"/>
+      <c r="B73" s="24"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="22"/>
-      <c r="B74" s="22"/>
+      <c r="A74" s="24"/>
+      <c r="B74" s="24"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="22"/>
-      <c r="B75" s="22"/>
+      <c r="A75" s="24"/>
+      <c r="B75" s="24"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="22"/>
-      <c r="B76" s="22"/>
+      <c r="A76" s="24"/>
+      <c r="B76" s="24"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="22"/>
-      <c r="B77" s="22"/>
+      <c r="A77" s="24"/>
+      <c r="B77" s="24"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="22"/>
-      <c r="B78" s="22"/>
+      <c r="A78" s="24"/>
+      <c r="B78" s="24"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="22"/>
-      <c r="B79" s="22"/>
+      <c r="A79" s="24"/>
+      <c r="B79" s="24"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="22"/>
-      <c r="B80" s="22"/>
+      <c r="A80" s="24"/>
+      <c r="B80" s="24"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="22"/>
-      <c r="B81" s="22"/>
+      <c r="A81" s="24"/>
+      <c r="B81" s="24"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="22"/>
-      <c r="B82" s="22"/>
+      <c r="A82" s="24"/>
+      <c r="B82" s="24"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="22"/>
-      <c r="B83" s="22"/>
+      <c r="A83" s="24"/>
+      <c r="B83" s="24"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="22"/>
-      <c r="B84" s="22"/>
+      <c r="A84" s="24"/>
+      <c r="B84" s="24"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="22"/>
-      <c r="B85" s="22"/>
+      <c r="A85" s="24"/>
+      <c r="B85" s="24"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="22"/>
-      <c r="B86" s="22"/>
+      <c r="A86" s="24"/>
+      <c r="B86" s="24"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="22"/>
-      <c r="B87" s="22"/>
+      <c r="A87" s="24"/>
+      <c r="B87" s="24"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="22"/>
-      <c r="B88" s="22"/>
+      <c r="A88" s="24"/>
+      <c r="B88" s="24"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="22"/>
-      <c r="B89" s="22"/>
+      <c r="A89" s="24"/>
+      <c r="B89" s="24"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="22"/>
-      <c r="B90" s="22"/>
+      <c r="A90" s="24"/>
+      <c r="B90" s="24"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="22"/>
-      <c r="B91" s="22"/>
+      <c r="A91" s="24"/>
+      <c r="B91" s="24"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="22"/>
-      <c r="B92" s="22"/>
+      <c r="A92" s="24"/>
+      <c r="B92" s="24"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="22"/>
-      <c r="B93" s="22"/>
+      <c r="A93" s="24"/>
+      <c r="B93" s="24"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="22"/>
-      <c r="B94" s="22"/>
+      <c r="A94" s="24"/>
+      <c r="B94" s="24"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="22"/>
-      <c r="B95" s="22"/>
+      <c r="A95" s="24"/>
+      <c r="B95" s="24"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="22"/>
-      <c r="B96" s="22"/>
+      <c r="A96" s="24"/>
+      <c r="B96" s="24"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="22"/>
-      <c r="B97" s="22"/>
+      <c r="A97" s="24"/>
+      <c r="B97" s="24"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="A98" s="22"/>
-      <c r="B98" s="22"/>
+      <c r="A98" s="24"/>
+      <c r="B98" s="24"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="22"/>
-      <c r="B99" s="22"/>
+      <c r="A99" s="24"/>
+      <c r="B99" s="24"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
-      <c r="A100" s="22"/>
-      <c r="B100" s="22"/>
+      <c r="A100" s="24"/>
+      <c r="B100" s="24"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="22"/>
-      <c r="B101" s="22"/>
+      <c r="A101" s="24"/>
+      <c r="B101" s="24"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
-      <c r="A102" s="22"/>
-      <c r="B102" s="22"/>
+      <c r="A102" s="24"/>
+      <c r="B102" s="24"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="22"/>
-      <c r="B103" s="22"/>
+      <c r="A103" s="24"/>
+      <c r="B103" s="24"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
-      <c r="A104" s="22"/>
-      <c r="B104" s="22"/>
+      <c r="A104" s="24"/>
+      <c r="B104" s="24"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="22"/>
-      <c r="B105" s="22"/>
+      <c r="A105" s="24"/>
+      <c r="B105" s="24"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="22"/>
-      <c r="B106" s="22"/>
+      <c r="A106" s="24"/>
+      <c r="B106" s="24"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="22"/>
-      <c r="B107" s="22"/>
+      <c r="A107" s="24"/>
+      <c r="B107" s="24"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="A108" s="22"/>
-      <c r="B108" s="22"/>
+      <c r="A108" s="24"/>
+      <c r="B108" s="24"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
-      <c r="A109" s="22"/>
-      <c r="B109" s="22"/>
+      <c r="A109" s="24"/>
+      <c r="B109" s="24"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="A110" s="22"/>
-      <c r="B110" s="22"/>
+      <c r="A110" s="24"/>
+      <c r="B110" s="24"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
-      <c r="A111" s="22"/>
-      <c r="B111" s="22"/>
+      <c r="A111" s="24"/>
+      <c r="B111" s="24"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
-      <c r="A112" s="22"/>
-      <c r="B112" s="22"/>
+      <c r="A112" s="24"/>
+      <c r="B112" s="24"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
-      <c r="A113" s="22"/>
-      <c r="B113" s="22"/>
+      <c r="A113" s="24"/>
+      <c r="B113" s="24"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
-      <c r="A114" s="22"/>
-      <c r="B114" s="22"/>
+      <c r="A114" s="24"/>
+      <c r="B114" s="24"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
-      <c r="A115" s="22"/>
-      <c r="B115" s="22"/>
+      <c r="A115" s="24"/>
+      <c r="B115" s="24"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="22"/>
-      <c r="B116" s="22"/>
+      <c r="A116" s="24"/>
+      <c r="B116" s="24"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
-      <c r="A117" s="22"/>
-      <c r="B117" s="22"/>
+      <c r="A117" s="24"/>
+      <c r="B117" s="24"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
-      <c r="A118" s="22"/>
-      <c r="B118" s="22"/>
+      <c r="A118" s="24"/>
+      <c r="B118" s="24"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
-      <c r="A119" s="22"/>
-      <c r="B119" s="22"/>
+      <c r="A119" s="24"/>
+      <c r="B119" s="24"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
-      <c r="A120" s="22"/>
-      <c r="B120" s="22"/>
+      <c r="A120" s="24"/>
+      <c r="B120" s="24"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
-      <c r="A121" s="22"/>
-      <c r="B121" s="22"/>
+      <c r="A121" s="24"/>
+      <c r="B121" s="24"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
-      <c r="A122" s="22"/>
-      <c r="B122" s="22"/>
+      <c r="A122" s="24"/>
+      <c r="B122" s="24"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
-      <c r="A123" s="22"/>
-      <c r="B123" s="22"/>
+      <c r="A123" s="24"/>
+      <c r="B123" s="24"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
-      <c r="A124" s="22"/>
-      <c r="B124" s="22"/>
+      <c r="A124" s="24"/>
+      <c r="B124" s="24"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
-      <c r="A125" s="22"/>
-      <c r="B125" s="22"/>
+      <c r="A125" s="24"/>
+      <c r="B125" s="24"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
-      <c r="A126" s="22"/>
-      <c r="B126" s="22"/>
+      <c r="A126" s="24"/>
+      <c r="B126" s="24"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
-      <c r="A127" s="22"/>
-      <c r="B127" s="22"/>
+      <c r="A127" s="24"/>
+      <c r="B127" s="24"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
-      <c r="A128" s="22"/>
-      <c r="B128" s="22"/>
+      <c r="A128" s="24"/>
+      <c r="B128" s="24"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
-      <c r="A129" s="22"/>
-      <c r="B129" s="22"/>
+      <c r="A129" s="24"/>
+      <c r="B129" s="24"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
-      <c r="A130" s="22"/>
-      <c r="B130" s="22"/>
+      <c r="A130" s="24"/>
+      <c r="B130" s="24"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
-      <c r="A131" s="22"/>
-      <c r="B131" s="22"/>
+      <c r="A131" s="24"/>
+      <c r="B131" s="24"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
-      <c r="A132" s="22"/>
-      <c r="B132" s="22"/>
+      <c r="A132" s="24"/>
+      <c r="B132" s="24"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
-      <c r="A133" s="22"/>
-      <c r="B133" s="22"/>
+      <c r="A133" s="24"/>
+      <c r="B133" s="24"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
-      <c r="A134" s="22"/>
-      <c r="B134" s="22"/>
+      <c r="A134" s="24"/>
+      <c r="B134" s="24"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
-      <c r="A135" s="22"/>
-      <c r="B135" s="22"/>
+      <c r="A135" s="24"/>
+      <c r="B135" s="24"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
-      <c r="A136" s="22"/>
-      <c r="B136" s="22"/>
+      <c r="A136" s="24"/>
+      <c r="B136" s="24"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
-      <c r="A137" s="22"/>
-      <c r="B137" s="22"/>
+      <c r="A137" s="24"/>
+      <c r="B137" s="24"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
-      <c r="A138" s="22"/>
-      <c r="B138" s="22"/>
+      <c r="A138" s="24"/>
+      <c r="B138" s="24"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
-      <c r="A139" s="22"/>
-      <c r="B139" s="22"/>
+      <c r="A139" s="24"/>
+      <c r="B139" s="24"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="A140" s="22"/>
-      <c r="B140" s="22"/>
+      <c r="A140" s="24"/>
+      <c r="B140" s="24"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
-      <c r="A141" s="22"/>
-      <c r="B141" s="22"/>
+      <c r="A141" s="24"/>
+      <c r="B141" s="24"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
-      <c r="A142" s="22"/>
-      <c r="B142" s="22"/>
+      <c r="A142" s="24"/>
+      <c r="B142" s="24"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
-      <c r="A143" s="22"/>
-      <c r="B143" s="22"/>
+      <c r="A143" s="24"/>
+      <c r="B143" s="24"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
-      <c r="A144" s="22"/>
-      <c r="B144" s="22"/>
+      <c r="A144" s="24"/>
+      <c r="B144" s="24"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="A145" s="22"/>
-      <c r="B145" s="22"/>
+      <c r="A145" s="24"/>
+      <c r="B145" s="24"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
-      <c r="A146" s="22"/>
-      <c r="B146" s="22"/>
+      <c r="A146" s="24"/>
+      <c r="B146" s="24"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
-      <c r="A147" s="22"/>
-      <c r="B147" s="22"/>
+      <c r="A147" s="24"/>
+      <c r="B147" s="24"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="A148" s="22"/>
-      <c r="B148" s="22"/>
+      <c r="A148" s="24"/>
+      <c r="B148" s="24"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="A149" s="22"/>
-      <c r="B149" s="22"/>
+      <c r="A149" s="24"/>
+      <c r="B149" s="24"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
-      <c r="A150" s="22"/>
-      <c r="B150" s="22"/>
+      <c r="A150" s="24"/>
+      <c r="B150" s="24"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="A151" s="22"/>
-      <c r="B151" s="22"/>
+      <c r="A151" s="24"/>
+      <c r="B151" s="24"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
-      <c r="A152" s="22"/>
-      <c r="B152" s="22"/>
+      <c r="A152" s="24"/>
+      <c r="B152" s="24"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="A153" s="22"/>
-      <c r="B153" s="22"/>
+      <c r="A153" s="24"/>
+      <c r="B153" s="24"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
-      <c r="A154" s="22"/>
-      <c r="B154" s="22"/>
+      <c r="A154" s="24"/>
+      <c r="B154" s="24"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
-      <c r="A155" s="22"/>
-      <c r="B155" s="22"/>
+      <c r="A155" s="24"/>
+      <c r="B155" s="24"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
-      <c r="A156" s="22"/>
-      <c r="B156" s="22"/>
+      <c r="A156" s="24"/>
+      <c r="B156" s="24"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
-      <c r="A157" s="22"/>
-      <c r="B157" s="22"/>
+      <c r="A157" s="24"/>
+      <c r="B157" s="24"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
-      <c r="A158" s="22"/>
-      <c r="B158" s="22"/>
+      <c r="A158" s="24"/>
+      <c r="B158" s="24"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
-      <c r="A159" s="22"/>
-      <c r="B159" s="22"/>
+      <c r="A159" s="24"/>
+      <c r="B159" s="24"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
-      <c r="A160" s="22"/>
-      <c r="B160" s="22"/>
+      <c r="A160" s="24"/>
+      <c r="B160" s="24"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
-      <c r="A161" s="22"/>
-      <c r="B161" s="22"/>
+      <c r="A161" s="24"/>
+      <c r="B161" s="24"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
-      <c r="A162" s="22"/>
-      <c r="B162" s="22"/>
+      <c r="A162" s="24"/>
+      <c r="B162" s="24"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
-      <c r="A163" s="22"/>
-      <c r="B163" s="22"/>
+      <c r="A163" s="24"/>
+      <c r="B163" s="24"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
-      <c r="A164" s="22"/>
-      <c r="B164" s="22"/>
+      <c r="A164" s="24"/>
+      <c r="B164" s="24"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
-      <c r="A165" s="22"/>
-      <c r="B165" s="22"/>
+      <c r="A165" s="24"/>
+      <c r="B165" s="24"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
-      <c r="A166" s="22"/>
-      <c r="B166" s="22"/>
+      <c r="A166" s="24"/>
+      <c r="B166" s="24"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
-      <c r="A167" s="22"/>
-      <c r="B167" s="22"/>
+      <c r="A167" s="24"/>
+      <c r="B167" s="24"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
-      <c r="A168" s="22"/>
-      <c r="B168" s="22"/>
+      <c r="A168" s="24"/>
+      <c r="B168" s="24"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
-      <c r="A169" s="22"/>
-      <c r="B169" s="22"/>
+      <c r="A169" s="24"/>
+      <c r="B169" s="24"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
-      <c r="A170" s="22"/>
-      <c r="B170" s="22"/>
+      <c r="A170" s="24"/>
+      <c r="B170" s="24"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
-      <c r="A171" s="22"/>
-      <c r="B171" s="22"/>
+      <c r="A171" s="24"/>
+      <c r="B171" s="24"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
-      <c r="A172" s="22"/>
-      <c r="B172" s="22"/>
+      <c r="A172" s="24"/>
+      <c r="B172" s="24"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
-      <c r="A173" s="22"/>
-      <c r="B173" s="22"/>
+      <c r="A173" s="24"/>
+      <c r="B173" s="24"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
-      <c r="A174" s="22"/>
-      <c r="B174" s="22"/>
+      <c r="A174" s="24"/>
+      <c r="B174" s="24"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
-      <c r="A175" s="22"/>
-      <c r="B175" s="22"/>
+      <c r="A175" s="24"/>
+      <c r="B175" s="24"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
-      <c r="A176" s="22"/>
-      <c r="B176" s="22"/>
+      <c r="A176" s="24"/>
+      <c r="B176" s="24"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
-      <c r="A177" s="22"/>
-      <c r="B177" s="22"/>
+      <c r="A177" s="24"/>
+      <c r="B177" s="24"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="A178" s="22"/>
-      <c r="B178" s="22"/>
+      <c r="A178" s="24"/>
+      <c r="B178" s="24"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
-      <c r="A179" s="22"/>
-      <c r="B179" s="22"/>
+      <c r="A179" s="24"/>
+      <c r="B179" s="24"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
-      <c r="A180" s="22"/>
-      <c r="B180" s="22"/>
+      <c r="A180" s="24"/>
+      <c r="B180" s="24"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
-      <c r="A181" s="22"/>
-      <c r="B181" s="22"/>
+      <c r="A181" s="24"/>
+      <c r="B181" s="24"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
-      <c r="A182" s="22"/>
-      <c r="B182" s="22"/>
+      <c r="A182" s="24"/>
+      <c r="B182" s="24"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
-      <c r="A183" s="22"/>
-      <c r="B183" s="22"/>
+      <c r="A183" s="24"/>
+      <c r="B183" s="24"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
-      <c r="A184" s="22"/>
-      <c r="B184" s="22"/>
+      <c r="A184" s="24"/>
+      <c r="B184" s="24"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
-      <c r="A185" s="22"/>
-      <c r="B185" s="22"/>
+      <c r="A185" s="24"/>
+      <c r="B185" s="24"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
-      <c r="A186" s="22"/>
-      <c r="B186" s="22"/>
+      <c r="A186" s="24"/>
+      <c r="B186" s="24"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
-      <c r="A187" s="22"/>
-      <c r="B187" s="22"/>
+      <c r="A187" s="24"/>
+      <c r="B187" s="24"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
-      <c r="A188" s="22"/>
-      <c r="B188" s="22"/>
+      <c r="A188" s="24"/>
+      <c r="B188" s="24"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
-      <c r="A189" s="22"/>
-      <c r="B189" s="22"/>
+      <c r="A189" s="24"/>
+      <c r="B189" s="24"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
-      <c r="A190" s="22"/>
-      <c r="B190" s="22"/>
+      <c r="A190" s="24"/>
+      <c r="B190" s="24"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
-      <c r="A191" s="22"/>
-      <c r="B191" s="22"/>
+      <c r="A191" s="24"/>
+      <c r="B191" s="24"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
-      <c r="A192" s="22"/>
-      <c r="B192" s="22"/>
+      <c r="A192" s="24"/>
+      <c r="B192" s="24"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
-      <c r="A193" s="22"/>
-      <c r="B193" s="22"/>
+      <c r="A193" s="24"/>
+      <c r="B193" s="24"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
-      <c r="A194" s="22"/>
-      <c r="B194" s="22"/>
+      <c r="A194" s="24"/>
+      <c r="B194" s="24"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
-      <c r="A195" s="22"/>
-      <c r="B195" s="22"/>
+      <c r="A195" s="24"/>
+      <c r="B195" s="24"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
-      <c r="A196" s="22"/>
-      <c r="B196" s="22"/>
+      <c r="A196" s="24"/>
+      <c r="B196" s="24"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
-      <c r="A197" s="22"/>
-      <c r="B197" s="22"/>
+      <c r="A197" s="24"/>
+      <c r="B197" s="24"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
-      <c r="A198" s="22"/>
-      <c r="B198" s="22"/>
+      <c r="A198" s="24"/>
+      <c r="B198" s="24"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
-      <c r="A199" s="22"/>
-      <c r="B199" s="22"/>
+      <c r="A199" s="24"/>
+      <c r="B199" s="24"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
-      <c r="A200" s="22"/>
-      <c r="B200" s="22"/>
+      <c r="A200" s="24"/>
+      <c r="B200" s="24"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
-      <c r="A201" s="22"/>
-      <c r="B201" s="22"/>
+      <c r="A201" s="24"/>
+      <c r="B201" s="24"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
-      <c r="A202" s="22"/>
-      <c r="B202" s="22"/>
+      <c r="A202" s="24"/>
+      <c r="B202" s="24"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
-      <c r="A203" s="22"/>
-      <c r="B203" s="22"/>
+      <c r="A203" s="24"/>
+      <c r="B203" s="24"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
-      <c r="A204" s="22"/>
-      <c r="B204" s="22"/>
+      <c r="A204" s="24"/>
+      <c r="B204" s="24"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
-      <c r="A205" s="22"/>
-      <c r="B205" s="22"/>
+      <c r="A205" s="24"/>
+      <c r="B205" s="24"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
-      <c r="A206" s="22"/>
-      <c r="B206" s="22"/>
+      <c r="A206" s="24"/>
+      <c r="B206" s="24"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
-      <c r="A207" s="22"/>
-      <c r="B207" s="22"/>
+      <c r="A207" s="24"/>
+      <c r="B207" s="24"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
-      <c r="A208" s="22"/>
-      <c r="B208" s="22"/>
+      <c r="A208" s="24"/>
+      <c r="B208" s="24"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
-      <c r="A209" s="22"/>
-      <c r="B209" s="22"/>
+      <c r="A209" s="24"/>
+      <c r="B209" s="24"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
-      <c r="A210" s="22"/>
-      <c r="B210" s="22"/>
+      <c r="A210" s="24"/>
+      <c r="B210" s="24"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
-      <c r="A211" s="22"/>
-      <c r="B211" s="22"/>
+      <c r="A211" s="24"/>
+      <c r="B211" s="24"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
-      <c r="A212" s="22"/>
-      <c r="B212" s="22"/>
+      <c r="A212" s="24"/>
+      <c r="B212" s="24"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
-      <c r="A213" s="22"/>
-      <c r="B213" s="22"/>
+      <c r="A213" s="24"/>
+      <c r="B213" s="24"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
-      <c r="A214" s="22"/>
-      <c r="B214" s="22"/>
+      <c r="A214" s="24"/>
+      <c r="B214" s="24"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
-      <c r="A215" s="22"/>
-      <c r="B215" s="22"/>
+      <c r="A215" s="24"/>
+      <c r="B215" s="24"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
-      <c r="A216" s="22"/>
-      <c r="B216" s="22"/>
+      <c r="A216" s="24"/>
+      <c r="B216" s="24"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
-      <c r="A217" s="22"/>
-      <c r="B217" s="22"/>
+      <c r="A217" s="24"/>
+      <c r="B217" s="24"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
-      <c r="A218" s="22"/>
-      <c r="B218" s="22"/>
+      <c r="A218" s="24"/>
+      <c r="B218" s="24"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
-      <c r="A219" s="22"/>
-      <c r="B219" s="22"/>
+      <c r="A219" s="24"/>
+      <c r="B219" s="24"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
-      <c r="A220" s="22"/>
-      <c r="B220" s="22"/>
+      <c r="A220" s="24"/>
+      <c r="B220" s="24"/>
     </row>
     <row r="221" ht="15.75" customHeight="1">
-      <c r="A221" s="22"/>
-      <c r="B221" s="22"/>
+      <c r="A221" s="24"/>
+      <c r="B221" s="24"/>
     </row>
     <row r="222" ht="15.75" customHeight="1">
-      <c r="A222" s="22"/>
-      <c r="B222" s="22"/>
+      <c r="A222" s="24"/>
+      <c r="B222" s="24"/>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="A223" s="22"/>
-      <c r="B223" s="22"/>
+      <c r="A223" s="24"/>
+      <c r="B223" s="24"/>
     </row>
     <row r="224" ht="15.75" customHeight="1">
-      <c r="A224" s="22"/>
-      <c r="B224" s="22"/>
+      <c r="A224" s="24"/>
+      <c r="B224" s="24"/>
     </row>
     <row r="225" ht="15.75" customHeight="1">
-      <c r="A225" s="22"/>
-      <c r="B225" s="22"/>
+      <c r="A225" s="24"/>
+      <c r="B225" s="24"/>
     </row>
     <row r="226" ht="15.75" customHeight="1">
-      <c r="A226" s="22"/>
-      <c r="B226" s="22"/>
+      <c r="A226" s="24"/>
+      <c r="B226" s="24"/>
     </row>
     <row r="227" ht="15.75" customHeight="1">
-      <c r="A227" s="22"/>
-      <c r="B227" s="22"/>
+      <c r="A227" s="24"/>
+      <c r="B227" s="24"/>
     </row>
     <row r="228" ht="15.75" customHeight="1">
-      <c r="A228" s="22"/>
-      <c r="B228" s="22"/>
+      <c r="A228" s="24"/>
+      <c r="B228" s="24"/>
     </row>
     <row r="229" ht="15.75" customHeight="1">
-      <c r="A229" s="22"/>
-      <c r="B229" s="22"/>
+      <c r="A229" s="24"/>
+      <c r="B229" s="24"/>
     </row>
     <row r="230" ht="15.75" customHeight="1">
-      <c r="A230" s="22"/>
-      <c r="B230" s="22"/>
+      <c r="A230" s="24"/>
+      <c r="B230" s="24"/>
     </row>
     <row r="231" ht="15.75" customHeight="1">
-      <c r="A231" s="22"/>
-      <c r="B231" s="22"/>
+      <c r="A231" s="24"/>
+      <c r="B231" s="24"/>
     </row>
     <row r="232" ht="15.75" customHeight="1">
-      <c r="A232" s="22"/>
-      <c r="B232" s="22"/>
+      <c r="A232" s="24"/>
+      <c r="B232" s="24"/>
     </row>
     <row r="233" ht="15.75" customHeight="1">
-      <c r="A233" s="22"/>
-      <c r="B233" s="22"/>
+      <c r="A233" s="24"/>
+      <c r="B233" s="24"/>
     </row>
     <row r="234" ht="15.75" customHeight="1">
-      <c r="A234" s="22"/>
-      <c r="B234" s="22"/>
+      <c r="A234" s="24"/>
+      <c r="B234" s="24"/>
     </row>
     <row r="235" ht="15.75" customHeight="1">
-      <c r="A235" s="22"/>
-      <c r="B235" s="22"/>
+      <c r="A235" s="24"/>
+      <c r="B235" s="24"/>
     </row>
     <row r="236" ht="15.75" customHeight="1">
-      <c r="A236" s="22"/>
-      <c r="B236" s="22"/>
+      <c r="A236" s="24"/>
+      <c r="B236" s="24"/>
     </row>
     <row r="237" ht="15.75" customHeight="1">
-      <c r="A237" s="22"/>
-      <c r="B237" s="22"/>
+      <c r="A237" s="24"/>
+      <c r="B237" s="24"/>
     </row>
     <row r="238" ht="15.75" customHeight="1">
-      <c r="A238" s="22"/>
-      <c r="B238" s="22"/>
+      <c r="A238" s="24"/>
+      <c r="B238" s="24"/>
     </row>
     <row r="239" ht="15.75" customHeight="1">
-      <c r="A239" s="22"/>
-      <c r="B239" s="22"/>
+      <c r="A239" s="24"/>
+      <c r="B239" s="24"/>
     </row>
     <row r="240" ht="15.75" customHeight="1">
-      <c r="A240" s="22"/>
-      <c r="B240" s="22"/>
+      <c r="A240" s="24"/>
+      <c r="B240" s="24"/>
     </row>
     <row r="241" ht="15.75" customHeight="1">
-      <c r="A241" s="22"/>
-      <c r="B241" s="22"/>
+      <c r="A241" s="24"/>
+      <c r="B241" s="24"/>
     </row>
     <row r="242" ht="15.75" customHeight="1">
-      <c r="A242" s="22"/>
-      <c r="B242" s="22"/>
+      <c r="A242" s="24"/>
+      <c r="B242" s="24"/>
     </row>
     <row r="243" ht="15.75" customHeight="1">
-      <c r="A243" s="22"/>
-      <c r="B243" s="22"/>
+      <c r="A243" s="24"/>
+      <c r="B243" s="24"/>
     </row>
     <row r="244" ht="15.75" customHeight="1">
-      <c r="A244" s="22"/>
-      <c r="B244" s="22"/>
+      <c r="A244" s="24"/>
+      <c r="B244" s="24"/>
     </row>
     <row r="245" ht="15.75" customHeight="1">
-      <c r="A245" s="22"/>
-      <c r="B245" s="22"/>
+      <c r="A245" s="24"/>
+      <c r="B245" s="24"/>
     </row>
     <row r="246" ht="15.75" customHeight="1">
-      <c r="A246" s="22"/>
-      <c r="B246" s="22"/>
+      <c r="A246" s="24"/>
+      <c r="B246" s="24"/>
     </row>
     <row r="247" ht="15.75" customHeight="1">
-      <c r="A247" s="22"/>
-      <c r="B247" s="22"/>
+      <c r="A247" s="24"/>
+      <c r="B247" s="24"/>
     </row>
     <row r="248" ht="15.75" customHeight="1">
-      <c r="A248" s="22"/>
-      <c r="B248" s="22"/>
+      <c r="A248" s="24"/>
+      <c r="B248" s="24"/>
     </row>
     <row r="249" ht="15.75" customHeight="1">
-      <c r="A249" s="22"/>
-      <c r="B249" s="22"/>
+      <c r="A249" s="24"/>
+      <c r="B249" s="24"/>
     </row>
     <row r="250" ht="15.75" customHeight="1">
-      <c r="A250" s="22"/>
-      <c r="B250" s="22"/>
+      <c r="A250" s="24"/>
+      <c r="B250" s="24"/>
     </row>
     <row r="251" ht="15.75" customHeight="1">
-      <c r="A251" s="22"/>
-      <c r="B251" s="22"/>
+      <c r="A251" s="24"/>
+      <c r="B251" s="24"/>
     </row>
     <row r="252" ht="15.75" customHeight="1">
-      <c r="A252" s="22"/>
-      <c r="B252" s="22"/>
+      <c r="A252" s="24"/>
+      <c r="B252" s="24"/>
     </row>
     <row r="253" ht="15.75" customHeight="1">
-      <c r="A253" s="22"/>
-      <c r="B253" s="22"/>
+      <c r="A253" s="24"/>
+      <c r="B253" s="24"/>
     </row>
     <row r="254" ht="15.75" customHeight="1">
-      <c r="A254" s="22"/>
-      <c r="B254" s="22"/>
+      <c r="A254" s="24"/>
+      <c r="B254" s="24"/>
     </row>
     <row r="255" ht="15.75" customHeight="1">
-      <c r="A255" s="22"/>
-      <c r="B255" s="22"/>
+      <c r="A255" s="24"/>
+      <c r="B255" s="24"/>
     </row>
     <row r="256" ht="15.75" customHeight="1">
-      <c r="A256" s="22"/>
-      <c r="B256" s="22"/>
+      <c r="A256" s="24"/>
+      <c r="B256" s="24"/>
     </row>
     <row r="257" ht="15.75" customHeight="1">
-      <c r="A257" s="22"/>
-      <c r="B257" s="22"/>
+      <c r="A257" s="24"/>
+      <c r="B257" s="24"/>
     </row>
     <row r="258" ht="15.75" customHeight="1">
-      <c r="A258" s="22"/>
-      <c r="B258" s="22"/>
+      <c r="A258" s="24"/>
+      <c r="B258" s="24"/>
     </row>
     <row r="259" ht="15.75" customHeight="1">
-      <c r="A259" s="22"/>
-      <c r="B259" s="22"/>
+      <c r="A259" s="24"/>
+      <c r="B259" s="24"/>
     </row>
     <row r="260" ht="15.75" customHeight="1">
-      <c r="A260" s="22"/>
-      <c r="B260" s="22"/>
+      <c r="A260" s="24"/>
+      <c r="B260" s="24"/>
     </row>
     <row r="261" ht="15.75" customHeight="1"/>
     <row r="262" ht="15.75" customHeight="1"/>
@@ -4914,49 +4958,49 @@
     <row r="4" ht="15.75" customHeight="1"/>
     <row r="5" ht="15.75" customHeight="1"/>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="25" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="I7" s="24" t="s">
+      <c r="I7" s="26" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="F8" s="25" t="s">
+      <c r="F8" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="27">
         <v>1043.0</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="27">
         <v>607.0</v>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="27">
         <v>58.1975</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="27">
         <v>957.0</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="27">
         <v>512.0</v>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="27">
         <v>53.5005</v>
       </c>
     </row>
@@ -5978,39 +6022,39 @@
     <row r="4" ht="15.75" customHeight="1"/>
     <row r="5" ht="15.75" customHeight="1"/>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="28" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="29">
         <v>2000.0</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="27">
-        <v>3431663.0</v>
+      <c r="G8" s="30">
+        <v>1.4888021E7</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="29">
         <v>55.95</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="29">
         <v>5670.635</v>
       </c>
     </row>

</xml_diff>